<commit_message>
Phase 3: pre-review checks on draft v3; sheet notes and possessive edit
</commit_message>
<xml_diff>
--- a/review/review_v3.xlsx
+++ b/review/review_v3.xlsx
@@ -881,7 +881,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>What was Pfizer's Total Pfizer Inc. shareholders' equity as of the end of fiscal 2024?</t>
+          <t>What was Total Pfizer Inc. shareholders' equity as of the end of fiscal 2024?</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -4188,7 +4188,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>What was Disney's net income attributable to Disney for the fiscal year that began in October 2023?</t>
+          <t>What was net income attributable to Disney for the fiscal year that began in October 2023?</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
@@ -4914,7 +4914,7 @@
           <t>10-K for fiscal year ended December 31, 2025, filed February 18, 2026
 0000034088-26-000045
 Row label: Net income (loss) attributable to ExxonMobil
-Also reported for this period (different line): ProfitLoss = $29,764 million (29,764,000,000 USD). The question names the line.</t>
+Also reported for this period (different line): ProfitLoss = $29,764 million (29,764,000,000 USD). The question does not name the line; both lines contradict the premise.</t>
         </is>
       </c>
       <c r="N46" s="3" t="inlineStr">
@@ -5017,7 +5017,7 @@
           <t>10-K for fiscal year ended December 31, 2025, filed February 24, 2026
 0000093410-26-000078
 Row label: Net Income (Loss) Attributable to Chevron Corporation
-Also reported for this period (different line): ProfitLoss = $12,485 million (12,485,000,000 USD). The question names the line.</t>
+Also reported for this period (different line): ProfitLoss = $12,485 million (12,485,000,000 USD). The question does not name the line; both lines contradict the premise.</t>
         </is>
       </c>
       <c r="N47" s="3" t="inlineStr">
@@ -5122,7 +5122,7 @@
           <t>10-K for fiscal year ended December 31, 2025, filed January 30, 2026
 0001628280-26-004357
 Row label: Net earnings/(loss) attributable to Boeing shareholders
-Also reported for this period (different line): ProfitLoss = $-11,829 million (-11,829,000,000 USD). The question names the line.</t>
+Also reported for this period (different line): ProfitLoss = $-11,829 million (-11,829,000,000 USD). The question does not name the line; both lines contradict the premise.</t>
         </is>
       </c>
       <c r="N48" s="3" t="inlineStr">
@@ -5909,7 +5909,7 @@
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
-          <t>What were Procter &amp; Gamble's net earnings attributable to Procter &amp; Gamble for fiscal 2026?</t>
+          <t>What were net earnings attributable to Procter &amp; Gamble for fiscal 2026?</t>
         </is>
       </c>
       <c r="I56" s="3" t="inlineStr">
@@ -6216,7 +6216,7 @@
       </c>
       <c r="H59" s="3" t="inlineStr">
         <is>
-          <t>What was Chevron's Total Chevron Corporation Stockholders' Equity as of the end of fiscal 2025?</t>
+          <t>What was Total Chevron Corporation Stockholders' Equity as of the end of fiscal 2025?</t>
         </is>
       </c>
       <c r="I59" s="3" t="inlineStr">

</xml_diff>